<commit_message>
update extension identity reliability 4933842965861ae29f75a044f64091e0f7836926
</commit_message>
<xml_diff>
--- a/ig/nr-add-def-ins-collection/CodeSystem-fr-core-fiabilite-identite.xlsx
+++ b/ig/nr-add-def-ins-collection/CodeSystem-fr-core-fiabilite-identite.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="83">
   <si>
     <t>Property</t>
   </si>
@@ -63,7 +63,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-10-16T15:07:43+00:00</t>
+    <t>2023-10-23T11:38:46+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -120,7 +120,7 @@
     <t>Count</t>
   </si>
   <si>
-    <t>19</t>
+    <t>21</t>
   </si>
   <si>
     <t>Level</t>
@@ -240,16 +240,28 @@
     <t>Homonyme détecté</t>
   </si>
   <si>
+    <t>INVA</t>
+  </si>
+  <si>
+    <t>Identité invalidée</t>
+  </si>
+  <si>
     <t>HOMA</t>
   </si>
   <si>
-    <t>Homonyme avéré</t>
-  </si>
-  <si>
-    <t>INVA</t>
-  </si>
-  <si>
-    <t>Identité invalidée</t>
+    <t>Homonyme avéré (attribut d'identité homonyme)</t>
+  </si>
+  <si>
+    <t>FICT</t>
+  </si>
+  <si>
+    <t>Identité fictive (attribut d'identité fictive)</t>
+  </si>
+  <si>
+    <t>DOUT</t>
+  </si>
+  <si>
+    <t>Identité douteuse (attribut d'identité douteuse)</t>
   </si>
 </sst>
 </file>
@@ -565,7 +577,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -810,6 +822,30 @@
       </c>
       <c r="D20" s="2"/>
     </row>
+    <row r="21">
+      <c r="A21" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B21" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="C21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="D21" s="2"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B22" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="C22" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="D22" s="2"/>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>